<commit_message>
Update return shipments data (auto)
</commit_message>
<xml_diff>
--- a/docs/data/returns_intransit.xlsx
+++ b/docs/data/returns_intransit.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -801,17 +801,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JVGLOTC0113619121</t>
+          <t>CY254064248DE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dhlparcel-nl</t>
+          <t>dhl-germany</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DHL Parcel NL</t>
+          <t>Deutsche Post DHL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6001659976</t>
+          <t>6001664166</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -833,18 +833,22 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-02T10:57:01+01:00</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>2026-02-05T14:01:00+01:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-03-02T10:58:15+00:00</t>
+          <t>2026-03-02T01:58:14+00:00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>JVGLOTC0113619121</t>
+          <t>CY254064248DE</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -856,17 +860,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>67721300002823</t>
+          <t>JJD149990121180200257</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hermes-de</t>
+          <t>dhlparcel-nl</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hermes Germany</t>
+          <t>DHL Parcel NL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -876,7 +880,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>6001662826</t>
+          <t>6001658918</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -888,14 +892,10 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-02-23T17:07:10+01:00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+          <t>2026-02-13T10:25:00+01:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>2026-03-02T01:58:14+00:00</t>
@@ -903,7 +903,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>67721300002823</t>
+          <t>JJD149990121180200257</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -915,17 +915,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CY429881982DE</t>
+          <t>YV6RE2R4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>dhl-germany</t>
+          <t>gls</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Deutsche Post DHL</t>
+          <t>GLS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>6001659732</t>
+          <t>6001658661</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -947,22 +947,22 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-02-16T13:00:00+01:00</t>
+          <t>2026-02-16T15:00:00+01:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>NL, Netherlands</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-03-02T01:58:14+00:00</t>
+          <t>2026-03-02T01:58:21+00:00</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>CY429881982DE</t>
+          <t>YV6RE2R4</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -974,17 +974,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>66045117400493</t>
+          <t>JVGLOTC0114408022</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hermes-de</t>
+          <t>dhlparcel-nl</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hermes Germany</t>
+          <t>DHL Parcel NL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>6001659078</t>
+          <t>6001659976</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1006,22 +1006,18 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-02-24T11:28:45+01:00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+          <t>2026-03-02T10:57:01+01:00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-03-02T01:58:14+00:00</t>
+          <t>2026-03-02T10:58:16+00:00</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>66045117400493</t>
+          <t>JVGLOTC0114408022</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1033,17 +1029,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>YV6RE2R4</t>
+          <t>JVGLOTC0113619121</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>gls</t>
+          <t>dhlparcel-nl</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GLS</t>
+          <t>DHL Parcel NL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1053,7 +1049,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>6001658661</t>
+          <t>6001659976</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1065,22 +1061,18 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-02-16T15:00:00+01:00</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>NL, Netherlands</t>
-        </is>
-      </c>
+          <t>2026-03-02T10:57:01+01:00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-03-02T01:58:21+00:00</t>
+          <t>2026-03-02T10:58:15+00:00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>YV6RE2R4</t>
+          <t>JVGLOTC0113619121</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1092,17 +1084,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>66051117400128</t>
+          <t>YV6RF1WX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>hermes-de</t>
+          <t>gls</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hermes Germany</t>
+          <t>GLS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1112,7 +1104,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>6001659012</t>
+          <t>6001658774</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1124,22 +1116,22 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-02-24T11:28:45+01:00</t>
+          <t>2026-02-26T16:00:00+01:00</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>NL, Netherlands</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-03-02T01:58:13+00:00</t>
+          <t>2026-03-02T01:58:20+00:00</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>66051117400128</t>
+          <t>YV6RF1WX</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1151,17 +1143,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JJD149990121180200257</t>
+          <t>CY429881982DE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>dhlparcel-nl</t>
+          <t>dhl-germany</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DHL Parcel NL</t>
+          <t>Deutsche Post DHL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1171,7 +1163,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6001658918</t>
+          <t>6001659732</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1183,10 +1175,14 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-02-13T10:25:00+01:00</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+          <t>2026-02-16T13:00:00+01:00</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>2026-03-02T01:58:14+00:00</t>
@@ -1194,301 +1190,10 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>JJD149990121180200257</t>
+          <t>CY429881982DE</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>YV6RF1WX</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>gls</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>GLS</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>6001658774</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>csv_importer</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-02-26T16:00:00+01:00</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>NL, Netherlands</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>2026-03-02T01:58:20+00:00</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>YV6RF1WX</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>66040117401334</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>hermes-de</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Hermes Germany</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>6001663147</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>csv_importer</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-02-26T11:26:31+01:00</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>2026-03-02T01:58:15+00:00</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>66040117401334</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>AA007903003763</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>brt-it-parcelid</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>BRT Bartolini(Parcel ID)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>6001662164</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>csv_importer</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2026-02-10T12:00:00+01:00</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>MILANO SEDRIANO (050)</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>2026-03-02T02:58:15+00:00</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>AA007903003763</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>JVGLOTC0114408022</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>dhlparcel-nl</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>DHL Parcel NL</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>6001659976</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>csv_importer</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-03-02T10:57:01+01:00</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>2026-03-02T10:58:16+00:00</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>JVGLOTC0114408022</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CY254064248DE</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>dhl-germany</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Deutsche Post DHL</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>6001664166</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>csv_importer</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2026-02-05T14:01:00+01:00</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>2026-03-02T01:58:14+00:00</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>CY254064248DE</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
         <is>
           <t>{}</t>
         </is>

</xml_diff>